<commit_message>
Fix logo and broker dropdown
</commit_message>
<xml_diff>
--- a/Healthx v Healthxclusive.xlsx
+++ b/Healthx v Healthxclusive.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasperhealthx/Desktop/AI Projects/Premium Summary /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{ABF5FC82-CFCE-2947-B84B-9A6EE3849301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12FC48FE-DF02-DC42-A5A3-95A1406B1950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{24387DBC-8823-354F-83E3-DFD1F4C62815}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="17400" xr2:uid="{24387DBC-8823-354F-83E3-DFD1F4C62815}"/>
   </bookViews>
   <sheets>
     <sheet name="Age Bands" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="22">
   <si>
     <t>Healthx</t>
   </si>
@@ -90,6 +90,18 @@
   </si>
   <si>
     <t>66 - 99</t>
+  </si>
+  <si>
+    <t>0 - 17</t>
+  </si>
+  <si>
+    <t>18 - 40</t>
+  </si>
+  <si>
+    <t>41 - 59</t>
+  </si>
+  <si>
+    <t>60 - 99</t>
   </si>
 </sst>
 </file>
@@ -499,7 +511,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88DE1501-E48A-8E48-B132-EF1A0BF9A0A8}">
-  <dimension ref="A2:C14"/>
+  <dimension ref="A2:E14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -507,7 +519,7 @@
     <col min="3" max="3" width="13.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -518,7 +530,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>3</v>
       </c>
@@ -528,8 +540,11 @@
       <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E3" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>4</v>
       </c>
@@ -539,8 +554,11 @@
       <c r="C4" s="2" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E4" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
@@ -550,8 +568,11 @@
       <c r="C5" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -561,8 +582,11 @@
       <c r="C6" s="2" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="E6" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>7</v>
       </c>
@@ -573,7 +597,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>8</v>
       </c>
@@ -584,7 +608,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
@@ -595,7 +619,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>10</v>
       </c>
@@ -606,7 +630,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>11</v>
       </c>
@@ -617,7 +641,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>12</v>
       </c>
@@ -628,7 +652,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>13</v>
       </c>
@@ -639,7 +663,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
         <v>14</v>
       </c>

</xml_diff>